<commit_message>
V0.3.0 - Rep CRSF_Serial integriert
</commit_message>
<xml_diff>
--- a/documentation/ESP32/Pinout.xlsx
+++ b/documentation/ESP32/Pinout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/roberttrampler/Projekte/LandRover/GIT_LandRover/LandRover_ESP32/documentation/ESP32/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EB0264-D682-CD47-AAD6-10D09DA28409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1186C6-2AD4-0A4C-918D-6DFEB0B44952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9720" yWindow="660" windowWidth="18960" windowHeight="19080" activeTab="1" xr2:uid="{1CF20767-7363-42F2-8642-5539791B45CC}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" activeTab="1" xr2:uid="{1CF20767-7363-42F2-8642-5539791B45CC}"/>
   </bookViews>
   <sheets>
     <sheet name="DOIT ESP32 DEVKIT V1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="218">
   <si>
     <t>pin1</t>
   </si>
@@ -716,12 +716,33 @@
   <si>
     <t>Rear / Brake lights</t>
   </si>
+  <si>
+    <t>Drehzahl VR</t>
+  </si>
+  <si>
+    <t>Drehzahl VL</t>
+  </si>
+  <si>
+    <t>Drehzahl HR</t>
+  </si>
+  <si>
+    <t>Drehzahl HL</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>UART</t>
+  </si>
+  <si>
+    <t>RC Communication</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -791,8 +812,16 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -895,6 +924,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -975,10 +1010,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1054,8 +1090,14 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2378,7 +2420,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:18">
-      <c r="B3" t="s">
+      <c r="B3" s="43" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2481,10 +2523,12 @@
       <c r="C9" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F9" s="3"/>
+      <c r="E9" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F9" s="42" t="s">
+        <v>215</v>
+      </c>
       <c r="G9" s="7" t="s">
         <v>44</v>
       </c>
@@ -2507,7 +2551,7 @@
       <c r="N9" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="O9" s="15" t="s">
+      <c r="O9" s="17" t="s">
         <v>100</v>
       </c>
       <c r="Q9" s="3" t="s">
@@ -2524,10 +2568,12 @@
       <c r="C10" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F10" s="3"/>
+      <c r="E10" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F10" s="42" t="s">
+        <v>215</v>
+      </c>
       <c r="G10" s="7" t="s">
         <v>45</v>
       </c>
@@ -2561,10 +2607,12 @@
       <c r="C11" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" s="3"/>
+      <c r="E11" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="F11" s="42" t="s">
+        <v>215</v>
+      </c>
       <c r="G11" s="7" t="s">
         <v>46</v>
       </c>
@@ -2602,10 +2650,12 @@
       <c r="C12" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F12" s="3"/>
+      <c r="E12" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="F12" s="42" t="s">
+        <v>215</v>
+      </c>
       <c r="G12" s="7" t="s">
         <v>47</v>
       </c>
@@ -2628,7 +2678,7 @@
       <c r="N12" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="O12" s="15" t="s">
+      <c r="O12" s="17" t="s">
         <v>100</v>
       </c>
       <c r="Q12" s="3" t="s">
@@ -2838,10 +2888,12 @@
       <c r="M17" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="N17" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="O17" s="3"/>
+      <c r="N17" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="O17" s="17" t="s">
+        <v>217</v>
+      </c>
       <c r="Q17" s="3" t="s">
         <v>99</v>
       </c>
@@ -2881,11 +2933,11 @@
       <c r="M18" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="N18" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="O18" s="14" t="s">
-        <v>114</v>
+      <c r="N18" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="O18" s="17" t="s">
+        <v>217</v>
       </c>
       <c r="Q18" s="3" t="s">
         <v>99</v>
@@ -2963,10 +3015,12 @@
       <c r="M20" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="N20" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="O20" s="3"/>
+      <c r="N20" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="O20" s="14" t="s">
+        <v>114</v>
+      </c>
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
     </row>
@@ -3159,6 +3213,7 @@
       <c r="N28" s="19"/>
     </row>
     <row r="29" spans="2:18">
+      <c r="E29" s="41"/>
       <c r="G29" s="8"/>
       <c r="H29" s="22" t="s">
         <v>73</v>
@@ -3222,8 +3277,11 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{8B83A467-D3BF-D742-9661-E11568AAEF69}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>